<commit_message>
changes to kape files latest
</commit_message>
<xml_diff>
--- a/dfir-installer-selector.xlsx
+++ b/dfir-installer-selector.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\dfir-installer-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E934526B-5AC9-4CE4-91CD-AC98BAB79CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4382862-96A0-4195-A24D-F0FB7A9A5907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="2310" windowWidth="16440" windowHeight="28320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="30960" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dfir-installer-selector" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="448">
   <si>
     <t>Tool</t>
   </si>
@@ -48,9 +48,6 @@
     <t>EncryptedDiskHunter</t>
   </si>
   <si>
-    <t>Exterro FTK Imager</t>
-  </si>
-  <si>
     <t>KAPE</t>
   </si>
   <si>
@@ -222,9 +219,6 @@
     <t>Testdisk</t>
   </si>
   <si>
-    <t>VSS_Carver.pyinfected</t>
-  </si>
-  <si>
     <t>CyberChef</t>
   </si>
   <si>
@@ -243,9 +237,6 @@
     <t>iDef Map Setup</t>
   </si>
   <si>
-    <t>JoakimSchichtTools</t>
-  </si>
-  <si>
     <t>OleTools</t>
   </si>
   <si>
@@ -393,12 +384,6 @@
     <t>Event Log Explorer Old</t>
   </si>
   <si>
-    <t>Event Log Explorer_Forensic</t>
-  </si>
-  <si>
-    <t>Event Log Explorer_Standard</t>
-  </si>
-  <si>
     <t>Partition-4DiagnosticParser</t>
   </si>
   <si>
@@ -666,9 +651,6 @@
     <t>Merlin</t>
   </si>
   <si>
-    <t>Metasploit Framework</t>
-  </si>
-  <si>
     <t>MicroBurst</t>
   </si>
   <si>
@@ -1038,9 +1020,6 @@
     <t>VSTOR</t>
   </si>
   <si>
-    <t>VMware Workstation</t>
-  </si>
-  <si>
     <t>VM</t>
   </si>
   <si>
@@ -1104,9 +1083,6 @@
     <t>DirectoryOpus</t>
   </si>
   <si>
-    <t>EDD</t>
-  </si>
-  <si>
     <t>EditPadLite</t>
   </si>
   <si>
@@ -1116,9 +1092,6 @@
     <t>hasher</t>
   </si>
   <si>
-    <t>KAPE-Big</t>
-  </si>
-  <si>
     <t>kernel-document-viewer</t>
   </si>
   <si>
@@ -1306,6 +1279,99 @@
   </si>
   <si>
     <t>VirtualBox</t>
+  </si>
+  <si>
+    <t>bulk_extractor-rec</t>
+  </si>
+  <si>
+    <t>Cain</t>
+  </si>
+  <si>
+    <t>DFIRPowerShellScripts</t>
+  </si>
+  <si>
+    <t>EVTXtract</t>
+  </si>
+  <si>
+    <t>Exterro FTK Imager 4</t>
+  </si>
+  <si>
+    <t>ExtractUsnJrnl</t>
+  </si>
+  <si>
+    <t>Grassmarlin</t>
+  </si>
+  <si>
+    <t>Indx2Csv</t>
+  </si>
+  <si>
+    <t>JoakimSchichtToolsOutdated</t>
+  </si>
+  <si>
+    <t>LogFileParser-Git</t>
+  </si>
+  <si>
+    <t>MakeContainer</t>
+  </si>
+  <si>
+    <t>MakeImage</t>
+  </si>
+  <si>
+    <t>MetaDiver</t>
+  </si>
+  <si>
+    <t>Mft2Csv</t>
+  </si>
+  <si>
+    <t>MicrosoftExtractorSuite</t>
+  </si>
+  <si>
+    <t>RawCopy</t>
+  </si>
+  <si>
+    <t>Registry-Write-Block</t>
+  </si>
+  <si>
+    <t>Registry-Write-Block-exe</t>
+  </si>
+  <si>
+    <t>ROADtools</t>
+  </si>
+  <si>
+    <t>RunAsTI</t>
+  </si>
+  <si>
+    <t>Secure2Csv</t>
+  </si>
+  <si>
+    <t>ShimCacheParser</t>
+  </si>
+  <si>
+    <t>UsnJrnl2Csv</t>
+  </si>
+  <si>
+    <t>VMware Workstation17</t>
+  </si>
+  <si>
+    <t>VSS_Carver</t>
+  </si>
+  <si>
+    <t>ICS</t>
+  </si>
+  <si>
+    <t>Jschicht</t>
+  </si>
+  <si>
+    <t>Acquisition</t>
+  </si>
+  <si>
+    <t>Recovery</t>
+  </si>
+  <si>
+    <t>UAL</t>
+  </si>
+  <si>
+    <t>Writeblock</t>
   </si>
 </sst>
 </file>
@@ -1370,10 +1436,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A1:B308" totalsRowShown="0">
-  <autoFilter ref="A1:B308" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B308">
-    <sortCondition ref="A1:A308"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A1:B301" totalsRowShown="0">
+  <autoFilter ref="A1:B301" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B301">
+    <sortCondition ref="A1:A301"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Tool"/>
@@ -1493,7 +1559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B384"/>
+  <dimension ref="A1:B400"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.109375" style="1" customWidth="1"/>
@@ -1510,82 +1576,82 @@
     </row>
     <row r="2" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -1598,418 +1664,418 @@
     </row>
     <row r="13" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -2030,826 +2096,826 @@
     </row>
     <row r="67" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>121</v>
+        <v>272</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>119</v>
+        <v>271</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>278</v>
+        <v>240</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>277</v>
+        <v>224</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>111</v>
+        <v>241</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>112</v>
+        <v>224</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>246</v>
+        <v>13</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>230</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>247</v>
+        <v>14</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>230</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>14</v>
+        <v>301</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>11</v>
+        <v>302</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>15</v>
+        <v>303</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>11</v>
+        <v>302</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>308</v>
+        <v>285</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>309</v>
+        <v>183</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>308</v>
+        <v>182</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>6</v>
+        <v>242</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>3</v>
+        <v>224</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>293</v>
+        <v>184</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>291</v>
+        <v>182</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>188</v>
+        <v>52</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>187</v>
+        <v>43</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>248</v>
+        <v>158</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>230</v>
+        <v>156</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>189</v>
+        <v>53</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>187</v>
+        <v>46</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>163</v>
+        <v>243</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>161</v>
+        <v>224</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>54</v>
+        <v>185</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>47</v>
+        <v>182</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>249</v>
+        <v>288</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>230</v>
+        <v>285</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>190</v>
+        <v>96</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>187</v>
+        <v>95</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>294</v>
+        <v>87</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>291</v>
+        <v>85</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>88</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>90</v>
+        <v>244</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>88</v>
+        <v>224</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>113</v>
+        <v>16</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>112</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>16</v>
+        <v>201</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>11</v>
+        <v>198</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>250</v>
+        <v>202</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>230</v>
+        <v>198</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>206</v>
+        <v>60</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>203</v>
+        <v>59</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>207</v>
+        <v>146</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>203</v>
+        <v>143</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>60</v>
+        <v>10</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>151</v>
+        <v>54</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>148</v>
+        <v>46</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>19</v>
+        <v>147</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>11</v>
+        <v>143</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>55</v>
+        <v>186</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>47</v>
+        <v>182</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>152</v>
+        <v>68</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>148</v>
+        <v>64</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
-        <v>191</v>
+        <v>245</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>187</v>
+        <v>224</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
-        <v>20</v>
+        <v>324</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>11</v>
+        <v>322</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
-        <v>70</v>
+        <v>246</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>66</v>
+        <v>224</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>330</v>
+        <v>248</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>328</v>
+        <v>224</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>252</v>
+        <v>20</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>230</v>
+        <v>10</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>254</v>
+        <v>289</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>230</v>
+        <v>285</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
-        <v>21</v>
+        <v>290</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>11</v>
+        <v>285</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
-        <v>279</v>
+        <v>187</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>277</v>
+        <v>182</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
-        <v>295</v>
+        <v>203</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>291</v>
+        <v>198</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
-        <v>296</v>
+        <v>204</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>291</v>
+        <v>198</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
-        <v>192</v>
+        <v>128</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>187</v>
+        <v>124</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
-        <v>208</v>
+        <v>6</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>203</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>209</v>
+        <v>74</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>203</v>
+        <v>73</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>133</v>
+        <v>325</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>129</v>
+        <v>322</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>75</v>
+        <v>291</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>76</v>
+        <v>285</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
-        <v>7</v>
+        <v>407</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>3</v>
+        <v>109</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
-        <v>77</v>
+        <v>408</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
-        <v>331</v>
+        <v>159</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>328</v>
+        <v>156</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
-        <v>297</v>
+        <v>216</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>291</v>
+        <v>217</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
-        <v>416</v>
+        <v>195</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>112</v>
+        <v>196</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
-        <v>417</v>
+        <v>97</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
-        <v>164</v>
+        <v>98</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>161</v>
+        <v>95</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
-        <v>222</v>
+        <v>160</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>223</v>
+        <v>156</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
-        <v>200</v>
+        <v>7</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>201</v>
+        <v>3</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
-        <v>100</v>
+        <v>205</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>98</v>
+        <v>198</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
-        <v>165</v>
+        <v>140</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
-        <v>210</v>
+        <v>161</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>203</v>
+        <v>156</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
-        <v>145</v>
+        <v>104</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>146</v>
+        <v>101</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
-        <v>78</v>
+        <v>334</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>76</v>
+        <v>332</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
-        <v>166</v>
+        <v>335</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>161</v>
+        <v>332</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
-        <v>153</v>
+        <v>336</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>148</v>
+        <v>332</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
-        <v>107</v>
+        <v>337</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>104</v>
+        <v>332</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
-        <v>341</v>
+        <v>206</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>339</v>
+        <v>198</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
-        <v>342</v>
+        <v>112</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>339</v>
+        <v>109</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
-        <v>343</v>
+        <v>21</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>339</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
-        <v>344</v>
+        <v>207</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>339</v>
+        <v>198</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
-        <v>212</v>
+        <v>249</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
-        <v>115</v>
+        <v>250</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>112</v>
+        <v>224</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
-        <v>22</v>
+        <v>188</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>11</v>
+        <v>182</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
-        <v>213</v>
+        <v>189</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>203</v>
+        <v>182</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
-        <v>214</v>
+        <v>162</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>203</v>
+        <v>156</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
-        <v>193</v>
+        <v>105</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>187</v>
+        <v>101</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
-        <v>167</v>
+        <v>218</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>161</v>
+        <v>217</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
-        <v>257</v>
+        <v>177</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>230</v>
+        <v>175</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
-        <v>258</v>
+        <v>22</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>230</v>
+        <v>10</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
-        <v>108</v>
+        <v>163</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>104</v>
+        <v>156</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
-        <v>195</v>
+        <v>69</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>187</v>
+        <v>64</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
-        <v>224</v>
+        <v>78</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>223</v>
+        <v>77</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
-        <v>182</v>
+        <v>79</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>180</v>
+        <v>77</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -2857,103 +2923,103 @@
         <v>23</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
-        <v>72</v>
+        <v>300</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>66</v>
+        <v>299</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
-        <v>82</v>
+        <v>319</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>80</v>
+        <v>320</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
-        <v>24</v>
+        <v>118</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
-        <v>306</v>
+        <v>219</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>305</v>
+        <v>217</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
-        <v>116</v>
+        <v>166</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>112</v>
+        <v>156</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
-        <v>325</v>
+        <v>167</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>326</v>
+        <v>156</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>119</v>
+        <v>156</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="182" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
-        <v>225</v>
+        <v>170</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>223</v>
+        <v>156</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -2961,695 +3027,695 @@
         <v>171</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="184" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
-        <v>172</v>
+        <v>24</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>161</v>
+        <v>10</v>
       </c>
     </row>
     <row r="185" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="186" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
-        <v>174</v>
+        <v>25</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>161</v>
+        <v>10</v>
       </c>
     </row>
     <row r="187" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
-        <v>175</v>
+        <v>292</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>161</v>
+        <v>285</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
-        <v>176</v>
+        <v>268</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>161</v>
+        <v>269</v>
       </c>
     </row>
     <row r="189" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
-        <v>25</v>
+        <v>274</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>11</v>
+        <v>271</v>
       </c>
     </row>
     <row r="190" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
-        <v>177</v>
+        <v>275</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>161</v>
+        <v>271</v>
       </c>
     </row>
     <row r="191" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
-        <v>26</v>
+        <v>253</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>11</v>
+        <v>224</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
-        <v>298</v>
+        <v>80</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>291</v>
+        <v>77</v>
       </c>
     </row>
     <row r="193" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
-        <v>274</v>
+        <v>81</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>275</v>
+        <v>77</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
-        <v>280</v>
+        <v>307</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>277</v>
+        <v>305</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
-        <v>281</v>
+        <v>308</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>277</v>
+        <v>305</v>
       </c>
     </row>
     <row r="196" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
-        <v>259</v>
+        <v>309</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>230</v>
+        <v>305</v>
       </c>
     </row>
     <row r="197" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
-        <v>83</v>
+        <v>310</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>80</v>
+        <v>305</v>
       </c>
     </row>
     <row r="198" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
-        <v>84</v>
+        <v>311</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>80</v>
+        <v>305</v>
       </c>
     </row>
     <row r="199" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>311</v>
+        <v>285</v>
       </c>
     </row>
     <row r="200" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
-        <v>314</v>
+        <v>114</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>311</v>
+        <v>109</v>
       </c>
     </row>
     <row r="201" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
-        <v>315</v>
+        <v>88</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>311</v>
+        <v>85</v>
       </c>
     </row>
     <row r="202" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
-        <v>316</v>
+        <v>254</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>311</v>
+        <v>224</v>
       </c>
     </row>
     <row r="203" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
-        <v>317</v>
+        <v>89</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>311</v>
+        <v>85</v>
       </c>
     </row>
     <row r="204" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
-        <v>299</v>
+        <v>90</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>291</v>
+        <v>85</v>
       </c>
     </row>
     <row r="205" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>112</v>
+        <v>85</v>
       </c>
     </row>
     <row r="206" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
-        <v>91</v>
+        <v>191</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>88</v>
+        <v>182</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
-        <v>260</v>
+        <v>209</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>230</v>
+        <v>198</v>
       </c>
     </row>
     <row r="208" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>88</v>
+        <v>10</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
-        <v>93</v>
+        <v>326</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>88</v>
+        <v>322</v>
       </c>
     </row>
     <row r="210" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
-        <v>94</v>
+        <v>255</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>88</v>
+        <v>224</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
-        <v>196</v>
+        <v>106</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>187</v>
+        <v>101</v>
       </c>
     </row>
     <row r="212" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
-        <v>215</v>
+        <v>122</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>203</v>
+        <v>120</v>
       </c>
     </row>
     <row r="213" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
-        <v>27</v>
+        <v>277</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>11</v>
+        <v>278</v>
       </c>
     </row>
     <row r="214" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>328</v>
+        <v>278</v>
       </c>
     </row>
     <row r="215" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>230</v>
+        <v>278</v>
       </c>
     </row>
     <row r="216" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
-        <v>109</v>
+        <v>281</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>104</v>
+        <v>278</v>
       </c>
     </row>
     <row r="217" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
-        <v>127</v>
+        <v>282</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>125</v>
+        <v>278</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
-        <v>283</v>
+        <v>312</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>284</v>
+        <v>305</v>
       </c>
     </row>
     <row r="219" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
-        <v>285</v>
+        <v>70</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>284</v>
+        <v>64</v>
       </c>
     </row>
     <row r="220" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
-        <v>286</v>
+        <v>71</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>284</v>
+        <v>64</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
-        <v>287</v>
+        <v>178</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>284</v>
+        <v>175</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
-        <v>288</v>
+        <v>256</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>284</v>
+        <v>224</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
-        <v>318</v>
+        <v>129</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>311</v>
+        <v>124</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
-        <v>73</v>
+        <v>210</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>66</v>
+        <v>198</v>
       </c>
     </row>
     <row r="225" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
-        <v>74</v>
+        <v>221</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>66</v>
+        <v>222</v>
       </c>
     </row>
     <row r="226" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
-        <v>183</v>
+        <v>223</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>180</v>
+        <v>222</v>
       </c>
     </row>
     <row r="227" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
-        <v>262</v>
+        <v>27</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>230</v>
+        <v>10</v>
       </c>
     </row>
     <row r="228" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
-        <v>134</v>
+        <v>294</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>129</v>
+        <v>285</v>
       </c>
     </row>
     <row r="229" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
-        <v>216</v>
+        <v>28</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>203</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
-        <v>227</v>
+        <v>149</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>228</v>
+        <v>143</v>
       </c>
     </row>
     <row r="231" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
-        <v>229</v>
+        <v>327</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>228</v>
+        <v>322</v>
       </c>
     </row>
     <row r="232" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="233" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
-        <v>300</v>
+        <v>130</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>291</v>
+        <v>124</v>
       </c>
     </row>
     <row r="234" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
-        <v>29</v>
+        <v>211</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>11</v>
+        <v>198</v>
       </c>
     </row>
     <row r="235" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A235" s="1" t="s">
-        <v>154</v>
+      <c r="A235" s="3" t="s">
+        <v>212</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>148</v>
+        <v>198</v>
       </c>
     </row>
     <row r="236" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
-        <v>333</v>
+        <v>61</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>328</v>
+        <v>59</v>
       </c>
     </row>
     <row r="237" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
-        <v>30</v>
+        <v>313</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>11</v>
+        <v>305</v>
       </c>
     </row>
     <row r="238" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
-        <v>135</v>
+        <v>173</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
     </row>
     <row r="239" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
-        <v>217</v>
+        <v>257</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
     </row>
     <row r="240" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A240" s="3" t="s">
-        <v>218</v>
+      <c r="A240" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>203</v>
+        <v>10</v>
       </c>
     </row>
     <row r="241" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
     </row>
     <row r="242" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
-        <v>319</v>
+        <v>258</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>311</v>
+        <v>224</v>
       </c>
     </row>
     <row r="243" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
-        <v>178</v>
+        <v>213</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>161</v>
+        <v>198</v>
       </c>
     </row>
     <row r="244" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
-        <v>263</v>
+        <v>31</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>230</v>
+        <v>10</v>
       </c>
     </row>
     <row r="245" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
-        <v>31</v>
+        <v>259</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>11</v>
+        <v>224</v>
       </c>
     </row>
     <row r="246" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A246" s="1" t="s">
-        <v>57</v>
+        <v>328</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>47</v>
+        <v>322</v>
       </c>
     </row>
     <row r="247" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
-        <v>264</v>
+        <v>32</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>230</v>
+        <v>10</v>
       </c>
     </row>
     <row r="248" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
-        <v>219</v>
+        <v>40</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>203</v>
+        <v>39</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
-        <v>32</v>
+        <v>314</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>11</v>
+        <v>305</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
-        <v>334</v>
+        <v>261</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>328</v>
+        <v>224</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B252" s="1" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="253" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="254" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
-        <v>320</v>
+        <v>34</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>311</v>
+        <v>10</v>
       </c>
     </row>
     <row r="255" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
-        <v>266</v>
+        <v>44</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>230</v>
+        <v>43</v>
       </c>
     </row>
     <row r="256" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
-        <v>267</v>
+        <v>283</v>
       </c>
       <c r="B256" s="1" t="s">
-        <v>230</v>
+        <v>278</v>
       </c>
     </row>
     <row r="257" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
-        <v>63</v>
+        <v>262</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>60</v>
+        <v>224</v>
       </c>
     </row>
     <row r="258" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
-        <v>34</v>
+        <v>151</v>
       </c>
       <c r="B258" s="1" t="s">
-        <v>11</v>
+        <v>152</v>
       </c>
     </row>
     <row r="259" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
-        <v>35</v>
+        <v>131</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>11</v>
+        <v>124</v>
       </c>
     </row>
     <row r="260" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
-        <v>45</v>
+        <v>132</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>44</v>
+        <v>124</v>
       </c>
     </row>
     <row r="261" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
-        <v>289</v>
+        <v>57</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>284</v>
+        <v>46</v>
       </c>
     </row>
     <row r="262" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
-        <v>268</v>
+        <v>295</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>230</v>
+        <v>285</v>
       </c>
     </row>
     <row r="263" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
-        <v>156</v>
+        <v>296</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>157</v>
+        <v>285</v>
       </c>
     </row>
     <row r="264" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
-        <v>136</v>
+        <v>297</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>129</v>
+        <v>285</v>
       </c>
     </row>
     <row r="265" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B265" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="266" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
-        <v>58</v>
+        <v>134</v>
       </c>
       <c r="B266" s="1" t="s">
-        <v>47</v>
+        <v>124</v>
       </c>
     </row>
     <row r="267" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
-        <v>301</v>
+        <v>136</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>291</v>
+        <v>124</v>
       </c>
     </row>
     <row r="268" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
-        <v>302</v>
+        <v>135</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>291</v>
+        <v>124</v>
       </c>
     </row>
     <row r="269" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
-        <v>303</v>
+        <v>137</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>291</v>
+        <v>124</v>
       </c>
     </row>
     <row r="270" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -3657,311 +3723,311 @@
         <v>138</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="271" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
-        <v>139</v>
+        <v>41</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>129</v>
+        <v>39</v>
       </c>
     </row>
     <row r="272" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
-        <v>141</v>
+        <v>107</v>
       </c>
       <c r="B272" s="1" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
     </row>
     <row r="273" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
-        <v>140</v>
+        <v>220</v>
       </c>
       <c r="B273" s="1" t="s">
-        <v>129</v>
+        <v>217</v>
       </c>
     </row>
     <row r="274" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
     </row>
     <row r="275" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
-        <v>143</v>
+        <v>93</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
     </row>
     <row r="276" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
-        <v>42</v>
+        <v>94</v>
       </c>
       <c r="B276" s="1" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
     </row>
     <row r="277" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
-        <v>110</v>
+        <v>179</v>
       </c>
       <c r="B277" s="1" t="s">
-        <v>104</v>
+        <v>175</v>
       </c>
     </row>
     <row r="278" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
-        <v>226</v>
+        <v>263</v>
       </c>
       <c r="B278" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="279" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
-        <v>95</v>
+        <v>8</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>88</v>
+        <v>3</v>
       </c>
     </row>
     <row r="280" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
-        <v>96</v>
+        <v>329</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>88</v>
+        <v>322</v>
       </c>
     </row>
     <row r="281" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
-        <v>97</v>
+        <v>192</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>88</v>
+        <v>182</v>
       </c>
     </row>
     <row r="282" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
-        <v>184</v>
+        <v>264</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>180</v>
+        <v>224</v>
       </c>
     </row>
     <row r="283" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
-        <v>336</v>
+        <v>214</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>337</v>
+        <v>198</v>
       </c>
     </row>
     <row r="284" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
-        <v>269</v>
+        <v>82</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>230</v>
+        <v>77</v>
       </c>
     </row>
     <row r="285" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
-        <v>9</v>
+        <v>315</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>3</v>
+        <v>305</v>
       </c>
     </row>
     <row r="286" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
-        <v>64</v>
+        <v>99</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>60</v>
+        <v>95</v>
       </c>
     </row>
     <row r="287" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
-        <v>335</v>
+        <v>139</v>
       </c>
       <c r="B287" s="1" t="s">
-        <v>328</v>
+        <v>124</v>
       </c>
     </row>
     <row r="288" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
-        <v>197</v>
+        <v>276</v>
       </c>
       <c r="B288" s="1" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
     </row>
     <row r="289" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
-        <v>270</v>
+        <v>338</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>230</v>
+        <v>332</v>
       </c>
     </row>
     <row r="290" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
-        <v>220</v>
+        <v>35</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>203</v>
+        <v>10</v>
       </c>
     </row>
     <row r="291" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
-        <v>85</v>
+        <v>340</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>80</v>
+        <v>332</v>
       </c>
     </row>
     <row r="292" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="B292" s="1" t="s">
-        <v>311</v>
+        <v>339</v>
+      </c>
+      <c r="B292" s="3" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="293" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
-        <v>102</v>
+        <v>193</v>
       </c>
       <c r="B293" s="1" t="s">
-        <v>98</v>
+        <v>182</v>
       </c>
     </row>
     <row r="294" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
-        <v>144</v>
+        <v>36</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
-        <v>282</v>
+        <v>194</v>
       </c>
       <c r="B295" s="1" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
-        <v>345</v>
+        <v>215</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
-        <v>36</v>
+        <v>153</v>
       </c>
       <c r="B297" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
-        <v>347</v>
+        <v>154</v>
       </c>
       <c r="B298" s="1" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="B299" s="3" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="B299" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A300" s="1" t="s">
-        <v>198</v>
+        <v>37</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="301" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A301" s="1" t="s">
-        <v>37</v>
+        <v>150</v>
       </c>
       <c r="B301" s="1" t="s">
-        <v>11</v>
+        <v>143</v>
       </c>
     </row>
     <row r="302" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A302" s="1" t="s">
-        <v>199</v>
+        <v>341</v>
       </c>
       <c r="B302" s="1" t="s">
-        <v>187</v>
+        <v>322</v>
       </c>
     </row>
     <row r="303" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A303" s="1" t="s">
-        <v>221</v>
+        <v>342</v>
       </c>
       <c r="B303" s="1" t="s">
-        <v>203</v>
+        <v>322</v>
       </c>
     </row>
     <row r="304" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
-        <v>158</v>
+        <v>343</v>
       </c>
       <c r="B304" s="1" t="s">
-        <v>157</v>
+        <v>182</v>
       </c>
     </row>
     <row r="305" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
-        <v>159</v>
+        <v>344</v>
       </c>
       <c r="B305" s="1" t="s">
-        <v>157</v>
+        <v>182</v>
       </c>
     </row>
     <row r="306" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
-        <v>86</v>
+        <v>345</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
     </row>
     <row r="307" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
-        <v>38</v>
+        <v>346</v>
       </c>
       <c r="B307" s="1" t="s">
-        <v>11</v>
+        <v>180</v>
       </c>
     </row>
     <row r="308" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
-        <v>155</v>
+        <v>347</v>
       </c>
       <c r="B308" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="309" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3969,7 +4035,7 @@
         <v>348</v>
       </c>
       <c r="B309" s="1" t="s">
-        <v>328</v>
+        <v>64</v>
       </c>
     </row>
     <row r="310" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3977,7 +4043,7 @@
         <v>349</v>
       </c>
       <c r="B310" s="1" t="s">
-        <v>328</v>
+        <v>64</v>
       </c>
     </row>
     <row r="311" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3985,7 +4051,7 @@
         <v>350</v>
       </c>
       <c r="B311" s="1" t="s">
-        <v>187</v>
+        <v>305</v>
       </c>
     </row>
     <row r="312" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3993,7 +4059,7 @@
         <v>351</v>
       </c>
       <c r="B312" s="1" t="s">
-        <v>187</v>
+        <v>305</v>
       </c>
     </row>
     <row r="313" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4001,7 +4067,7 @@
         <v>352</v>
       </c>
       <c r="B313" s="1" t="s">
-        <v>40</v>
+        <v>180</v>
       </c>
     </row>
     <row r="314" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4009,7 +4075,7 @@
         <v>353</v>
       </c>
       <c r="B314" s="1" t="s">
-        <v>185</v>
+        <v>10</v>
       </c>
     </row>
     <row r="315" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4017,7 +4083,7 @@
         <v>354</v>
       </c>
       <c r="B315" s="1" t="s">
-        <v>148</v>
+        <v>10</v>
       </c>
     </row>
     <row r="316" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4025,7 +4091,7 @@
         <v>355</v>
       </c>
       <c r="B316" s="1" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
     </row>
     <row r="317" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4033,7 +4099,7 @@
         <v>356</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
     </row>
     <row r="318" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4041,7 +4107,7 @@
         <v>357</v>
       </c>
       <c r="B318" s="1" t="s">
-        <v>311</v>
+        <v>10</v>
       </c>
     </row>
     <row r="319" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4049,7 +4115,7 @@
         <v>358</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>185</v>
+        <v>10</v>
       </c>
     </row>
     <row r="320" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4057,7 +4123,7 @@
         <v>359</v>
       </c>
       <c r="B320" s="1" t="s">
-        <v>311</v>
+        <v>10</v>
       </c>
     </row>
     <row r="321" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4065,7 +4131,7 @@
         <v>360</v>
       </c>
       <c r="B321" s="1" t="s">
-        <v>185</v>
+        <v>10</v>
       </c>
     </row>
     <row r="322" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4073,7 +4139,7 @@
         <v>361</v>
       </c>
       <c r="B322" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="323" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4081,7 +4147,7 @@
         <v>362</v>
       </c>
       <c r="B323" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="324" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4089,7 +4155,7 @@
         <v>363</v>
       </c>
       <c r="B324" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="325" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4097,7 +4163,7 @@
         <v>364</v>
       </c>
       <c r="B325" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="326" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4105,7 +4171,7 @@
         <v>365</v>
       </c>
       <c r="B326" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="327" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4113,7 +4179,7 @@
         <v>366</v>
       </c>
       <c r="B327" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="328" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4121,7 +4187,7 @@
         <v>367</v>
       </c>
       <c r="B328" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="329" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4129,7 +4195,7 @@
         <v>368</v>
       </c>
       <c r="B329" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="330" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4137,7 +4203,7 @@
         <v>369</v>
       </c>
       <c r="B330" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="331" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4145,7 +4211,7 @@
         <v>370</v>
       </c>
       <c r="B331" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="332" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4153,7 +4219,7 @@
         <v>371</v>
       </c>
       <c r="B332" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="333" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4161,7 +4227,7 @@
         <v>372</v>
       </c>
       <c r="B333" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="334" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4169,7 +4235,7 @@
         <v>373</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="335" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4177,7 +4243,7 @@
         <v>374</v>
       </c>
       <c r="B335" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="336" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4185,7 +4251,7 @@
         <v>375</v>
       </c>
       <c r="B336" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="337" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4193,7 +4259,7 @@
         <v>376</v>
       </c>
       <c r="B337" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="338" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4201,7 +4267,7 @@
         <v>377</v>
       </c>
       <c r="B338" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="339" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4209,7 +4275,7 @@
         <v>378</v>
       </c>
       <c r="B339" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="340" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4217,7 +4283,7 @@
         <v>379</v>
       </c>
       <c r="B340" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="341" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4225,7 +4291,7 @@
         <v>380</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="342" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4233,7 +4299,7 @@
         <v>381</v>
       </c>
       <c r="B342" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="343" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4241,7 +4307,7 @@
         <v>382</v>
       </c>
       <c r="B343" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="344" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4249,7 +4315,7 @@
         <v>383</v>
       </c>
       <c r="B344" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="345" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4257,7 +4323,7 @@
         <v>384</v>
       </c>
       <c r="B345" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="346" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4265,7 +4331,7 @@
         <v>385</v>
       </c>
       <c r="B346" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="347" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4273,7 +4339,7 @@
         <v>386</v>
       </c>
       <c r="B347" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="348" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4281,7 +4347,7 @@
         <v>387</v>
       </c>
       <c r="B348" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="349" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4289,7 +4355,7 @@
         <v>388</v>
       </c>
       <c r="B349" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="350" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4297,7 +4363,7 @@
         <v>389</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="351" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4305,7 +4371,7 @@
         <v>390</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="352" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4313,7 +4379,7 @@
         <v>391</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="353" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4321,7 +4387,7 @@
         <v>392</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="354" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4329,7 +4395,7 @@
         <v>393</v>
       </c>
       <c r="B354" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="355" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4337,7 +4403,7 @@
         <v>394</v>
       </c>
       <c r="B355" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="356" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4345,7 +4411,7 @@
         <v>395</v>
       </c>
       <c r="B356" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="357" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4353,7 +4419,7 @@
         <v>396</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="358" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4361,7 +4427,7 @@
         <v>397</v>
       </c>
       <c r="B358" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="359" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4369,7 +4435,7 @@
         <v>398</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>11</v>
+        <v>180</v>
       </c>
     </row>
     <row r="360" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4377,7 +4443,7 @@
         <v>399</v>
       </c>
       <c r="B360" s="1" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
     </row>
     <row r="361" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4385,7 +4451,7 @@
         <v>400</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>11</v>
+        <v>224</v>
       </c>
     </row>
     <row r="362" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4393,7 +4459,7 @@
         <v>401</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>11</v>
+        <v>182</v>
       </c>
     </row>
     <row r="363" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4401,7 +4467,7 @@
         <v>402</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="364" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4409,7 +4475,7 @@
         <v>403</v>
       </c>
       <c r="B364" s="1" t="s">
-        <v>11</v>
+        <v>180</v>
       </c>
     </row>
     <row r="365" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4417,7 +4483,7 @@
         <v>404</v>
       </c>
       <c r="B365" s="1" t="s">
-        <v>11</v>
+        <v>101</v>
       </c>
     </row>
     <row r="366" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4425,7 +4491,7 @@
         <v>405</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>11</v>
+        <v>332</v>
       </c>
     </row>
     <row r="367" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4433,79 +4499,79 @@
         <v>406</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>11</v>
+        <v>305</v>
       </c>
     </row>
     <row r="368" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A368" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>185</v>
+        <v>95</v>
       </c>
     </row>
     <row r="369" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A369" s="1" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
     </row>
     <row r="370" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A370" s="1" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>230</v>
+        <v>182</v>
       </c>
     </row>
     <row r="371" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A371" s="1" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="372" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A372" s="1" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="373" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A373" s="1" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>185</v>
+        <v>224</v>
       </c>
     </row>
     <row r="374" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A374" s="1" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>104</v>
+        <v>322</v>
       </c>
     </row>
     <row r="375" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A375" s="1" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B375" s="1" t="s">
-        <v>339</v>
+        <v>322</v>
       </c>
     </row>
     <row r="376" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A376" s="1" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>311</v>
+        <v>332</v>
       </c>
     </row>
     <row r="377" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4513,7 +4579,7 @@
         <v>418</v>
       </c>
       <c r="B377" s="1" t="s">
-        <v>98</v>
+        <v>224</v>
       </c>
     </row>
     <row r="378" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4521,7 +4587,7 @@
         <v>419</v>
       </c>
       <c r="B378" s="1" t="s">
-        <v>11</v>
+        <v>224</v>
       </c>
     </row>
     <row r="379" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4529,7 +4595,7 @@
         <v>420</v>
       </c>
       <c r="B379" s="1" t="s">
-        <v>187</v>
+        <v>445</v>
       </c>
     </row>
     <row r="380" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4537,7 +4603,7 @@
         <v>421</v>
       </c>
       <c r="B380" s="1" t="s">
-        <v>187</v>
+        <v>444</v>
       </c>
     </row>
     <row r="381" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4545,7 +4611,7 @@
         <v>422</v>
       </c>
       <c r="B381" s="1" t="s">
-        <v>11</v>
+        <v>443</v>
       </c>
     </row>
     <row r="382" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4553,7 +4619,7 @@
         <v>423</v>
       </c>
       <c r="B382" s="1" t="s">
-        <v>230</v>
+        <v>442</v>
       </c>
     </row>
     <row r="383" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4561,7 +4627,7 @@
         <v>424</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>328</v>
+        <v>443</v>
       </c>
     </row>
     <row r="384" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4569,7 +4635,135 @@
         <v>425</v>
       </c>
       <c r="B384" s="1" t="s">
-        <v>328</v>
+        <v>443</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A385" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B385" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A386" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B386" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A387" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B387" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A388" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B388" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A389" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B389" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A390" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B390" s="1" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A391" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B391" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A392" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B392" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A393" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B393" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A394" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="B394" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A395" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B395" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A396" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="B396" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A397" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B397" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A398" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="B398" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A399" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B399" s="1" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A400" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="B400" s="1" t="s">
+        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Tool list and categories
</commit_message>
<xml_diff>
--- a/dfir-installer-selector.xlsx
+++ b/dfir-installer-selector.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\dfir-installer-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4382862-96A0-4195-A24D-F0FB7A9A5907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B231AF5F-8A89-4D2D-BCD1-BC0CB8D15545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="30960" windowHeight="12120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="416">
   <si>
     <t>Tool</t>
   </si>
@@ -249,9 +249,6 @@
     <t>KANSA-PP</t>
   </si>
   <si>
-    <t>Custom</t>
-  </si>
-  <si>
     <t>kapexplaso-pp</t>
   </si>
   <si>
@@ -315,9 +312,6 @@
     <t>VisualStudioEnterprise2022</t>
   </si>
   <si>
-    <t>Driver</t>
-  </si>
-  <si>
     <t>GIGABYTEControlCenter</t>
   </si>
   <si>
@@ -390,9 +384,6 @@
     <t>ArtiFast</t>
   </si>
   <si>
-    <t>Forensic Suits</t>
-  </si>
-  <si>
     <t>Autopsy</t>
   </si>
   <si>
@@ -453,9 +444,6 @@
     <t>Maltego</t>
   </si>
   <si>
-    <t>Inteligence</t>
-  </si>
-  <si>
     <t>Capa</t>
   </si>
   <si>
@@ -486,9 +474,6 @@
     <t>Ubuntu2204</t>
   </si>
   <si>
-    <t>Linux</t>
-  </si>
-  <si>
     <t>WSL</t>
   </si>
   <si>
@@ -570,9 +555,6 @@
     <t>VLC</t>
   </si>
   <si>
-    <t>Misc</t>
-  </si>
-  <si>
     <t>Apimonitor</t>
   </si>
   <si>
@@ -618,9 +600,6 @@
     <t>Logfileparser</t>
   </si>
   <si>
-    <t>NTFS Tools</t>
-  </si>
-  <si>
     <t>adconnectdump</t>
   </si>
   <si>
@@ -828,9 +807,6 @@
     <t>ChocolateyGUI</t>
   </si>
   <si>
-    <t>Package Manager</t>
-  </si>
-  <si>
     <t>DockerDesktop</t>
   </si>
   <si>
@@ -843,9 +819,6 @@
     <t>BuildTools</t>
   </si>
   <si>
-    <t>Recommended</t>
-  </si>
-  <si>
     <t>Everything</t>
   </si>
   <si>
@@ -927,18 +900,12 @@
     <t>DeepSound</t>
   </si>
   <si>
-    <t>Stegano</t>
-  </si>
-  <si>
     <t>openstego</t>
   </si>
   <si>
     <t>Explorer Suite</t>
   </si>
   <si>
-    <t>Suite</t>
-  </si>
-  <si>
     <t>Explorersuite</t>
   </si>
   <si>
@@ -981,18 +948,12 @@
     <t>Cmder</t>
   </si>
   <si>
-    <t>Terminal</t>
-  </si>
-  <si>
     <t>Cygwin</t>
   </si>
   <si>
     <t>parseusbs</t>
   </si>
   <si>
-    <t>USB Forensics</t>
-  </si>
-  <si>
     <t>Cutter</t>
   </si>
   <si>
@@ -1020,9 +981,6 @@
     <t>VSTOR</t>
   </si>
   <si>
-    <t>VM</t>
-  </si>
-  <si>
     <t>DataDump</t>
   </si>
   <si>
@@ -1077,9 +1035,6 @@
     <t>Comae-Toolkit</t>
   </si>
   <si>
-    <t>dfir-installer</t>
-  </si>
-  <si>
     <t>DirectoryOpus</t>
   </si>
   <si>
@@ -1095,9 +1050,6 @@
     <t>kernel-document-viewer</t>
   </si>
   <si>
-    <t>kernel-emlx-viewer</t>
-  </si>
-  <si>
     <t>kernel-sql-backup-recovery</t>
   </si>
   <si>
@@ -1125,9 +1077,6 @@
     <t>kernelbkf-viewer</t>
   </si>
   <si>
-    <t>kernelbulkimageresizer</t>
-  </si>
-  <si>
     <t>kernelcalcdemo</t>
   </si>
   <si>
@@ -1140,24 +1089,15 @@
     <t>kernelemlviewer</t>
   </si>
   <si>
-    <t>kernelexchange-edb-viewer</t>
-  </si>
-  <si>
     <t>kernelexchangetogroup64</t>
   </si>
   <si>
-    <t>Kernelforexchangetonotes</t>
-  </si>
-  <si>
     <t>kernelfreekernelolmviewer</t>
   </si>
   <si>
     <t>kernelfreekerneloutlookpstreporter</t>
   </si>
   <si>
-    <t>kernelgrptonotes</t>
-  </si>
-  <si>
     <t>kernelimpressdemo</t>
   </si>
   <si>
@@ -1167,33 +1107,9 @@
     <t>kernelmboxviewer</t>
   </si>
   <si>
-    <t>kernelmdb-viewer</t>
-  </si>
-  <si>
     <t>kernelmdf-viewer</t>
   </si>
   <si>
-    <t>kernelnotestogrp</t>
-  </si>
-  <si>
-    <t>kernelnotestopdfdemo</t>
-  </si>
-  <si>
-    <t>kernelnsf-viewer</t>
-  </si>
-  <si>
-    <t>kernelnst-viewer</t>
-  </si>
-  <si>
-    <t>kernelNucleus-IE-Password</t>
-  </si>
-  <si>
-    <t>kernelNucleus-Kernel-DBX</t>
-  </si>
-  <si>
-    <t>kernelNucleus-Kernel-Excel</t>
-  </si>
-  <si>
     <t>kernelNucleus-Kernel-IncrediMail-Demo</t>
   </si>
   <si>
@@ -1203,9 +1119,6 @@
     <t>kernelNucleus-MSN-Password</t>
   </si>
   <si>
-    <t>kernelNucleus-PST-Password-Demo</t>
-  </si>
-  <si>
     <t>kerneloetonotes</t>
   </si>
   <si>
@@ -1356,22 +1269,13 @@
     <t>VSS_Carver</t>
   </si>
   <si>
-    <t>ICS</t>
-  </si>
-  <si>
-    <t>Jschicht</t>
-  </si>
-  <si>
-    <t>Acquisition</t>
-  </si>
-  <si>
     <t>Recovery</t>
   </si>
   <si>
-    <t>UAL</t>
-  </si>
-  <si>
     <t>Writeblock</t>
+  </si>
+  <si>
+    <t>NTFS</t>
   </si>
 </sst>
 </file>
@@ -1436,10 +1340,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A1:B301" totalsRowShown="0">
-  <autoFilter ref="A1:B301" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B301">
-    <sortCondition ref="A1:A301"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A1:B385" totalsRowShown="0">
+  <autoFilter ref="A1:B385" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B385">
+    <sortCondition ref="B1:B385"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Tool"/>
@@ -1559,10 +1463,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B400"/>
+  <dimension ref="A1:B385"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1576,127 +1480,127 @@
     </row>
     <row r="2" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>123</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>124</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>100</v>
+        <v>317</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>101</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>197</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>198</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>155</v>
+        <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>156</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>174</v>
+        <v>392</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>175</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>225</v>
+        <v>125</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>224</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>181</v>
+        <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>182</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>226</v>
+        <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>224</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>227</v>
+        <v>402</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>228</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>224</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>2</v>
+        <v>381</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>120</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>230</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>224</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>229</v>
+        <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>224</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>121</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>120</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>10</v>
@@ -1704,63 +1608,63 @@
     </row>
     <row r="18" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>231</v>
+        <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>224</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>284</v>
+        <v>338</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>285</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>286</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>285</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>199</v>
+        <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>198</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>270</v>
+        <v>350</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>271</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>11</v>
+        <v>339</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>10</v>
@@ -1768,151 +1672,151 @@
     </row>
     <row r="26" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>200</v>
+        <v>354</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>198</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>102</v>
+        <v>358</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>101</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>232</v>
+        <v>359</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>224</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>142</v>
+        <v>342</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>143</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>144</v>
+        <v>341</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>143</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>103</v>
+        <v>346</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>101</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>265</v>
+        <v>400</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>266</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>317</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>304</v>
+        <v>24</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>305</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>306</v>
+        <v>25</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>305</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>321</v>
+        <v>26</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>322</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>63</v>
+        <v>373</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>64</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>318</v>
+        <v>27</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>317</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>331</v>
+        <v>409</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>332</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>10</v>
@@ -1920,143 +1824,143 @@
     </row>
     <row r="45" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>233</v>
+        <v>30</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>224</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>234</v>
+        <v>31</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>224</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>298</v>
+        <v>32</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>299</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>145</v>
+        <v>34</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>143</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>125</v>
+        <v>256</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>124</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>235</v>
+        <v>35</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>224</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>64</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>157</v>
+        <v>37</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>156</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>236</v>
+        <v>331</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>224</v>
+        <v>39</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>237</v>
+        <v>38</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>224</v>
+        <v>39</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>238</v>
+        <v>40</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>224</v>
+        <v>39</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>267</v>
+        <v>41</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>266</v>
+        <v>39</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>323</v>
+        <v>42</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>322</v>
+        <v>43</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>126</v>
+        <v>52</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>124</v>
+        <v>43</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>127</v>
+        <v>44</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>124</v>
+        <v>43</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>239</v>
+        <v>45</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>224</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>46</v>
@@ -2064,191 +1968,191 @@
     </row>
     <row r="63" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>333</v>
+        <v>48</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>332</v>
+        <v>46</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>176</v>
+        <v>237</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>175</v>
+        <v>46</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>116</v>
+        <v>46</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>117</v>
+        <v>55</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>116</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>272</v>
+        <v>56</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>271</v>
+        <v>46</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>108</v>
+        <v>57</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>109</v>
+        <v>46</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>224</v>
+        <v>59</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>241</v>
+        <v>61</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>224</v>
+        <v>59</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>14</v>
+        <v>412</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>301</v>
+        <v>117</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>302</v>
+        <v>64</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>303</v>
+        <v>118</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>302</v>
+        <v>64</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>287</v>
+        <v>334</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>285</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>183</v>
+        <v>63</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>182</v>
+        <v>64</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>242</v>
+        <v>65</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>224</v>
+        <v>64</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>184</v>
+        <v>66</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>182</v>
+        <v>64</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>158</v>
+        <v>68</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>156</v>
+        <v>64</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>53</v>
+        <v>370</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>64</v>
@@ -2256,23 +2160,23 @@
     </row>
     <row r="87" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>243</v>
+        <v>119</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>224</v>
+        <v>64</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>185</v>
+        <v>70</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>182</v>
+        <v>64</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>64</v>
@@ -2280,1471 +2184,1471 @@
     </row>
     <row r="90" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>288</v>
+        <v>255</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>285</v>
+        <v>64</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>10</v>
+        <v>76</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>244</v>
+        <v>81</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>224</v>
+        <v>76</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>16</v>
+        <v>82</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>10</v>
+        <v>76</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>201</v>
+        <v>83</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>198</v>
+        <v>84</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>202</v>
+        <v>85</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>198</v>
+        <v>84</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>146</v>
+        <v>88</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>143</v>
+        <v>84</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>10</v>
+        <v>84</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>10</v>
+        <v>84</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>46</v>
+        <v>84</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>46</v>
+        <v>84</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>147</v>
+        <v>375</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>143</v>
+        <v>84</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>186</v>
+        <v>93</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>182</v>
+        <v>84</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>19</v>
+        <v>98</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>64</v>
+        <v>99</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
-        <v>245</v>
+        <v>101</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>224</v>
+        <v>99</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
-        <v>324</v>
+        <v>102</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>322</v>
+        <v>99</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
-        <v>246</v>
+        <v>103</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>224</v>
+        <v>99</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>247</v>
+        <v>104</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>224</v>
+        <v>99</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>248</v>
+        <v>105</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>224</v>
+        <v>99</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>20</v>
+        <v>106</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>10</v>
+        <v>107</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
-        <v>273</v>
+        <v>108</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>271</v>
+        <v>107</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>289</v>
+        <v>352</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>285</v>
+        <v>107</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
-        <v>290</v>
+        <v>378</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>285</v>
+        <v>107</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
-        <v>187</v>
+        <v>379</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>182</v>
+        <v>107</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
-        <v>203</v>
+        <v>109</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>198</v>
+        <v>107</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
-        <v>204</v>
+        <v>110</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>198</v>
+        <v>107</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
-        <v>6</v>
+        <v>113</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>3</v>
+        <v>114</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>73</v>
+        <v>114</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>325</v>
+        <v>116</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>322</v>
+        <v>114</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>291</v>
+        <v>120</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>285</v>
+        <v>121</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
-        <v>407</v>
+        <v>220</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
-        <v>408</v>
+        <v>122</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>156</v>
+        <v>121</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
-        <v>216</v>
+        <v>124</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>217</v>
+        <v>121</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
-        <v>195</v>
+        <v>126</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>196</v>
+        <v>121</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
-        <v>97</v>
+        <v>128</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>95</v>
+        <v>121</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>95</v>
+        <v>121</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
-        <v>160</v>
+        <v>130</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>156</v>
+        <v>121</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
-        <v>7</v>
+        <v>131</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>3</v>
+        <v>121</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
-        <v>205</v>
+        <v>133</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>198</v>
+        <v>121</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>73</v>
+        <v>121</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
-        <v>161</v>
+        <v>136</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>156</v>
+        <v>121</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
-        <v>104</v>
+        <v>140</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>101</v>
+        <v>139</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>332</v>
+        <v>139</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
-        <v>335</v>
+        <v>141</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>332</v>
+        <v>139</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
-        <v>336</v>
+        <v>142</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>332</v>
+        <v>139</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
-        <v>337</v>
+        <v>143</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>332</v>
+        <v>139</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
-        <v>206</v>
+        <v>144</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>198</v>
+        <v>139</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>109</v>
+        <v>139</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
-        <v>21</v>
+        <v>146</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>10</v>
+        <v>139</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
-        <v>207</v>
+        <v>150</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>198</v>
+        <v>151</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>198</v>
+        <v>151</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
-        <v>249</v>
+        <v>221</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>224</v>
+        <v>151</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
-        <v>250</v>
+        <v>223</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>224</v>
+        <v>151</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
-        <v>188</v>
+        <v>222</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
-        <v>189</v>
+        <v>277</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
-        <v>162</v>
+        <v>226</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
-        <v>251</v>
+        <v>227</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>224</v>
+        <v>151</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>252</v>
+        <v>228</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>224</v>
+        <v>151</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
-        <v>105</v>
+        <v>152</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>101</v>
+        <v>151</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>190</v>
+        <v>229</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>217</v>
+        <v>151</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
-        <v>177</v>
+        <v>231</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
-        <v>22</v>
+        <v>232</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>10</v>
+        <v>151</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
-        <v>163</v>
+        <v>233</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
-        <v>69</v>
+        <v>234</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>64</v>
+        <v>151</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
-        <v>78</v>
+        <v>291</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>77</v>
+        <v>151</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
-        <v>79</v>
+        <v>292</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>77</v>
+        <v>151</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
-        <v>23</v>
+        <v>278</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>10</v>
+        <v>151</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
-        <v>164</v>
+        <v>235</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
-        <v>300</v>
+        <v>153</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>299</v>
+        <v>151</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
-        <v>113</v>
+        <v>236</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>109</v>
+        <v>151</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>320</v>
+        <v>151</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
-        <v>118</v>
+        <v>280</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>116</v>
+        <v>151</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
-        <v>165</v>
+        <v>281</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
-        <v>219</v>
+        <v>282</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>217</v>
+        <v>151</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
-        <v>168</v>
+        <v>74</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="182" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="184" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
-        <v>24</v>
+        <v>159</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>10</v>
+        <v>151</v>
       </c>
     </row>
     <row r="185" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="186" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
-        <v>25</v>
+        <v>161</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>10</v>
+        <v>151</v>
       </c>
     </row>
     <row r="187" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
-        <v>292</v>
+        <v>162</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>285</v>
+        <v>151</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
-        <v>268</v>
+        <v>163</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>269</v>
+        <v>151</v>
       </c>
     </row>
     <row r="189" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
-        <v>274</v>
+        <v>164</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>271</v>
+        <v>151</v>
       </c>
     </row>
     <row r="190" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
-        <v>275</v>
+        <v>165</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>271</v>
+        <v>151</v>
       </c>
     </row>
     <row r="191" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
-        <v>253</v>
+        <v>166</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>224</v>
+        <v>151</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
-        <v>80</v>
+        <v>167</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>77</v>
+        <v>151</v>
       </c>
     </row>
     <row r="193" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
-        <v>81</v>
+        <v>283</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>77</v>
+        <v>151</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
-        <v>307</v>
+        <v>284</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>305</v>
+        <v>151</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
-        <v>308</v>
+        <v>285</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>305</v>
+        <v>151</v>
       </c>
     </row>
     <row r="196" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
-        <v>309</v>
+        <v>168</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>305</v>
+        <v>151</v>
       </c>
     </row>
     <row r="197" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
-        <v>310</v>
+        <v>286</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>305</v>
+        <v>151</v>
       </c>
     </row>
     <row r="198" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
-        <v>311</v>
+        <v>287</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>305</v>
+        <v>151</v>
       </c>
     </row>
     <row r="199" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>285</v>
+        <v>151</v>
       </c>
     </row>
     <row r="200" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
-        <v>114</v>
+        <v>169</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>109</v>
+        <v>170</v>
       </c>
     </row>
     <row r="201" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
-        <v>88</v>
+        <v>171</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>85</v>
+        <v>170</v>
       </c>
     </row>
     <row r="202" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
-        <v>254</v>
+        <v>172</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>224</v>
+        <v>170</v>
       </c>
     </row>
     <row r="203" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
-        <v>89</v>
+        <v>173</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>85</v>
+        <v>170</v>
       </c>
     </row>
     <row r="204" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
-        <v>90</v>
+        <v>174</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>85</v>
+        <v>170</v>
       </c>
     </row>
     <row r="205" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
-        <v>91</v>
+        <v>329</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>85</v>
+        <v>176</v>
       </c>
     </row>
     <row r="206" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
-        <v>191</v>
+        <v>330</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
-        <v>209</v>
+        <v>175</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
     </row>
     <row r="208" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
-        <v>26</v>
+        <v>382</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>10</v>
+        <v>176</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
-        <v>326</v>
+        <v>383</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>322</v>
+        <v>176</v>
       </c>
     </row>
     <row r="210" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
-        <v>255</v>
+        <v>177</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>224</v>
+        <v>176</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>101</v>
+        <v>176</v>
       </c>
     </row>
     <row r="212" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
-        <v>122</v>
+        <v>179</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>120</v>
+        <v>176</v>
       </c>
     </row>
     <row r="213" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
-        <v>277</v>
+        <v>394</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>278</v>
+        <v>176</v>
       </c>
     </row>
     <row r="214" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
-        <v>279</v>
+        <v>180</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>278</v>
+        <v>176</v>
       </c>
     </row>
     <row r="215" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
-        <v>280</v>
+        <v>181</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>278</v>
+        <v>176</v>
       </c>
     </row>
     <row r="216" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
-        <v>281</v>
+        <v>182</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>278</v>
+        <v>176</v>
       </c>
     </row>
     <row r="217" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
-        <v>282</v>
+        <v>183</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>278</v>
+        <v>176</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
-        <v>312</v>
+        <v>184</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>305</v>
+        <v>176</v>
       </c>
     </row>
     <row r="219" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
-        <v>70</v>
+        <v>185</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>64</v>
+        <v>176</v>
       </c>
     </row>
     <row r="220" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
-        <v>71</v>
+        <v>372</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>64</v>
+        <v>176</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
-        <v>256</v>
+        <v>187</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>224</v>
+        <v>176</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
-        <v>129</v>
+        <v>188</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>124</v>
+        <v>176</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
-        <v>210</v>
+        <v>393</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>198</v>
+        <v>415</v>
       </c>
     </row>
     <row r="225" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
-        <v>221</v>
+        <v>395</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>222</v>
+        <v>415</v>
       </c>
     </row>
     <row r="226" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
-        <v>223</v>
+        <v>384</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>222</v>
+        <v>415</v>
       </c>
     </row>
     <row r="227" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
-        <v>27</v>
+        <v>396</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>10</v>
+        <v>415</v>
       </c>
     </row>
     <row r="228" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
-        <v>294</v>
+        <v>189</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>285</v>
+        <v>415</v>
       </c>
     </row>
     <row r="229" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
-        <v>28</v>
+        <v>397</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>10</v>
+        <v>415</v>
       </c>
     </row>
     <row r="230" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
-        <v>149</v>
+        <v>401</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>143</v>
+        <v>415</v>
       </c>
     </row>
     <row r="231" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
-        <v>327</v>
+        <v>403</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>322</v>
+        <v>415</v>
       </c>
     </row>
     <row r="232" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
-        <v>29</v>
+        <v>410</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>10</v>
+        <v>415</v>
       </c>
     </row>
     <row r="233" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>124</v>
+        <v>191</v>
       </c>
     </row>
     <row r="234" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="235" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A235" s="3" t="s">
-        <v>212</v>
+      <c r="A235" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="236" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
-        <v>61</v>
+        <v>194</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>59</v>
+        <v>191</v>
       </c>
     </row>
     <row r="237" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
-        <v>313</v>
+        <v>195</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>305</v>
+        <v>191</v>
       </c>
     </row>
     <row r="238" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
     </row>
     <row r="239" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
-        <v>257</v>
+        <v>198</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>224</v>
+        <v>191</v>
       </c>
     </row>
     <row r="240" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A240" s="1" t="s">
-        <v>30</v>
+        <v>199</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>10</v>
+        <v>191</v>
       </c>
     </row>
     <row r="241" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
-        <v>56</v>
+        <v>200</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>46</v>
+        <v>191</v>
       </c>
     </row>
     <row r="242" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
-        <v>258</v>
+        <v>201</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>224</v>
+        <v>191</v>
       </c>
     </row>
     <row r="243" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="244" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
-        <v>31</v>
+        <v>203</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>10</v>
+        <v>191</v>
       </c>
     </row>
     <row r="245" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
-        <v>259</v>
+        <v>204</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>224</v>
+        <v>191</v>
       </c>
     </row>
     <row r="246" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A246" s="1" t="s">
-        <v>328</v>
+      <c r="A246" s="3" t="s">
+        <v>205</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>322</v>
+        <v>191</v>
       </c>
     </row>
     <row r="247" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
-        <v>32</v>
+        <v>206</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>10</v>
+        <v>191</v>
       </c>
     </row>
     <row r="248" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
-        <v>40</v>
+        <v>207</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>39</v>
+        <v>191</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
-        <v>314</v>
+        <v>208</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>305</v>
+        <v>191</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
-        <v>260</v>
+        <v>209</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>224</v>
+        <v>210</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
-        <v>261</v>
+        <v>211</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>224</v>
+        <v>210</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
-        <v>62</v>
+        <v>212</v>
       </c>
       <c r="B252" s="1" t="s">
-        <v>59</v>
+        <v>210</v>
       </c>
     </row>
     <row r="253" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
-        <v>33</v>
+        <v>213</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>10</v>
+        <v>210</v>
       </c>
     </row>
     <row r="254" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
-        <v>34</v>
+        <v>137</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>10</v>
+        <v>215</v>
       </c>
     </row>
     <row r="255" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
-        <v>44</v>
+        <v>214</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>43</v>
+        <v>215</v>
       </c>
     </row>
     <row r="256" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
-        <v>283</v>
+        <v>216</v>
       </c>
       <c r="B256" s="1" t="s">
-        <v>278</v>
+        <v>215</v>
       </c>
     </row>
     <row r="257" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
-        <v>262</v>
+        <v>219</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="258" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
-        <v>151</v>
+        <v>224</v>
       </c>
       <c r="B258" s="1" t="s">
-        <v>152</v>
+        <v>217</v>
       </c>
     </row>
     <row r="259" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
-        <v>131</v>
+        <v>225</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="260" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
-        <v>132</v>
+        <v>389</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="261" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
-        <v>57</v>
+        <v>289</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>46</v>
+        <v>217</v>
       </c>
     </row>
     <row r="262" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
-        <v>295</v>
+        <v>390</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>285</v>
+        <v>217</v>
       </c>
     </row>
     <row r="263" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
-        <v>296</v>
+        <v>238</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>285</v>
+        <v>217</v>
       </c>
     </row>
     <row r="264" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
-        <v>297</v>
+        <v>239</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>285</v>
+        <v>217</v>
       </c>
     </row>
     <row r="265" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
-        <v>133</v>
+        <v>240</v>
       </c>
       <c r="B265" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="266" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
-        <v>134</v>
+        <v>241</v>
       </c>
       <c r="B266" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="267" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
-        <v>136</v>
+        <v>264</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="268" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
-        <v>135</v>
+        <v>347</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="269" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
-        <v>137</v>
+        <v>348</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="270" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
-        <v>138</v>
+        <v>349</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
     </row>
     <row r="271" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
-        <v>41</v>
+        <v>351</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>39</v>
+        <v>217</v>
       </c>
     </row>
     <row r="272" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
-        <v>107</v>
+        <v>353</v>
       </c>
       <c r="B272" s="1" t="s">
-        <v>101</v>
+        <v>217</v>
       </c>
     </row>
     <row r="273" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
-        <v>220</v>
+        <v>355</v>
       </c>
       <c r="B273" s="1" t="s">
         <v>217</v>
@@ -3752,1029 +3656,909 @@
     </row>
     <row r="274" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
-        <v>92</v>
+        <v>356</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>85</v>
+        <v>217</v>
       </c>
     </row>
     <row r="275" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
-        <v>93</v>
+        <v>357</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>85</v>
+        <v>217</v>
       </c>
     </row>
     <row r="276" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
-        <v>94</v>
+        <v>360</v>
       </c>
       <c r="B276" s="1" t="s">
-        <v>85</v>
+        <v>217</v>
       </c>
     </row>
     <row r="277" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
-        <v>179</v>
+        <v>361</v>
       </c>
       <c r="B277" s="1" t="s">
-        <v>175</v>
+        <v>217</v>
       </c>
     </row>
     <row r="278" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
-        <v>263</v>
+        <v>363</v>
       </c>
       <c r="B278" s="1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="279" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
-        <v>8</v>
+        <v>364</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>3</v>
+        <v>217</v>
       </c>
     </row>
     <row r="280" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
-        <v>329</v>
+        <v>365</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
-        <v>192</v>
+        <v>366</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
-        <v>214</v>
+        <v>344</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
-        <v>82</v>
+        <v>367</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
-        <v>315</v>
+        <v>368</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
-        <v>99</v>
+        <v>369</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
-        <v>139</v>
+        <v>398</v>
       </c>
       <c r="B287" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
-        <v>276</v>
+        <v>399</v>
       </c>
       <c r="B288" s="1" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
-        <v>338</v>
+        <v>242</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
-        <v>35</v>
+        <v>243</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
-        <v>340</v>
+        <v>244</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="B292" s="3" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>245</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
-        <v>193</v>
+        <v>290</v>
       </c>
       <c r="B293" s="1" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
-        <v>36</v>
+        <v>246</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>10</v>
+        <v>217</v>
       </c>
     </row>
     <row r="295" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="B295" s="1" t="s">
-        <v>182</v>
+        <v>217</v>
       </c>
     </row>
     <row r="296" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
-        <v>215</v>
+        <v>248</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
     </row>
     <row r="297" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
-        <v>153</v>
+        <v>406</v>
       </c>
       <c r="B297" s="1" t="s">
-        <v>152</v>
+        <v>217</v>
       </c>
     </row>
     <row r="298" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
-        <v>154</v>
+        <v>407</v>
       </c>
       <c r="B298" s="1" t="s">
-        <v>152</v>
+        <v>217</v>
       </c>
     </row>
     <row r="299" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
-        <v>83</v>
+        <v>249</v>
       </c>
       <c r="B299" s="1" t="s">
-        <v>77</v>
+        <v>217</v>
       </c>
     </row>
     <row r="300" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A300" s="1" t="s">
-        <v>37</v>
+        <v>408</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>10</v>
+        <v>217</v>
       </c>
     </row>
     <row r="301" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A301" s="1" t="s">
-        <v>150</v>
+        <v>385</v>
       </c>
       <c r="B301" s="1" t="s">
-        <v>143</v>
+        <v>217</v>
       </c>
     </row>
     <row r="302" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A302" s="1" t="s">
-        <v>341</v>
+        <v>250</v>
       </c>
       <c r="B302" s="1" t="s">
-        <v>322</v>
+        <v>217</v>
       </c>
     </row>
     <row r="303" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A303" s="1" t="s">
-        <v>342</v>
+        <v>251</v>
       </c>
       <c r="B303" s="1" t="s">
-        <v>322</v>
+        <v>217</v>
       </c>
     </row>
     <row r="304" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
-        <v>343</v>
+        <v>252</v>
       </c>
       <c r="B304" s="1" t="s">
-        <v>182</v>
+        <v>217</v>
       </c>
     </row>
     <row r="305" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
-        <v>344</v>
+        <v>254</v>
       </c>
       <c r="B305" s="1" t="s">
-        <v>182</v>
+        <v>217</v>
       </c>
     </row>
     <row r="306" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
-        <v>345</v>
+        <v>257</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>39</v>
+        <v>217</v>
       </c>
     </row>
     <row r="307" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
-        <v>346</v>
+        <v>72</v>
       </c>
       <c r="B307" s="1" t="s">
-        <v>180</v>
+        <v>261</v>
       </c>
     </row>
     <row r="308" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
-        <v>347</v>
+        <v>73</v>
       </c>
       <c r="B308" s="1" t="s">
-        <v>143</v>
+        <v>261</v>
       </c>
     </row>
     <row r="309" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
-        <v>348</v>
+        <v>371</v>
       </c>
       <c r="B309" s="1" t="s">
-        <v>64</v>
+        <v>261</v>
       </c>
     </row>
     <row r="310" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A310" s="1" t="s">
-        <v>349</v>
+        <v>260</v>
       </c>
       <c r="B310" s="1" t="s">
-        <v>64</v>
+        <v>261</v>
       </c>
     </row>
     <row r="311" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A311" s="1" t="s">
-        <v>350</v>
+        <v>127</v>
       </c>
       <c r="B311" s="1" t="s">
-        <v>305</v>
+        <v>261</v>
       </c>
     </row>
     <row r="312" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A312" s="1" t="s">
-        <v>351</v>
+        <v>391</v>
       </c>
       <c r="B312" s="1" t="s">
-        <v>305</v>
+        <v>114</v>
       </c>
     </row>
     <row r="313" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A313" s="1" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="B313" s="1" t="s">
-        <v>180</v>
+        <v>413</v>
       </c>
     </row>
     <row r="314" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A314" s="1" t="s">
-        <v>353</v>
+        <v>340</v>
       </c>
       <c r="B314" s="1" t="s">
-        <v>10</v>
+        <v>413</v>
       </c>
     </row>
     <row r="315" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A315" s="1" t="s">
-        <v>354</v>
+        <v>345</v>
       </c>
       <c r="B315" s="1" t="s">
-        <v>10</v>
+        <v>413</v>
       </c>
     </row>
     <row r="316" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A316" s="1" t="s">
-        <v>355</v>
+        <v>268</v>
       </c>
       <c r="B316" s="1" t="s">
-        <v>10</v>
+        <v>269</v>
       </c>
     </row>
     <row r="317" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A317" s="1" t="s">
-        <v>356</v>
+        <v>270</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>10</v>
+        <v>269</v>
       </c>
     </row>
     <row r="318" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A318" s="1" t="s">
-        <v>357</v>
+        <v>271</v>
       </c>
       <c r="B318" s="1" t="s">
-        <v>10</v>
+        <v>269</v>
       </c>
     </row>
     <row r="319" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A319" s="1" t="s">
-        <v>358</v>
+        <v>272</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>10</v>
+        <v>269</v>
       </c>
     </row>
     <row r="320" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A320" s="1" t="s">
-        <v>359</v>
+        <v>273</v>
       </c>
       <c r="B320" s="1" t="s">
-        <v>10</v>
+        <v>269</v>
       </c>
     </row>
     <row r="321" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A321" s="1" t="s">
-        <v>360</v>
+        <v>274</v>
       </c>
       <c r="B321" s="1" t="s">
-        <v>10</v>
+        <v>269</v>
       </c>
     </row>
     <row r="322" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A322" s="1" t="s">
-        <v>361</v>
+        <v>275</v>
       </c>
       <c r="B322" s="1" t="s">
-        <v>10</v>
+        <v>276</v>
       </c>
     </row>
     <row r="323" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A323" s="1" t="s">
-        <v>362</v>
+        <v>308</v>
       </c>
       <c r="B323" s="1" t="s">
-        <v>10</v>
+        <v>276</v>
       </c>
     </row>
     <row r="324" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A324" s="1" t="s">
-        <v>363</v>
+        <v>279</v>
       </c>
       <c r="B324" s="1" t="s">
-        <v>10</v>
+        <v>276</v>
       </c>
     </row>
     <row r="325" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A325" s="1" t="s">
-        <v>364</v>
+        <v>313</v>
       </c>
       <c r="B325" s="1" t="s">
-        <v>10</v>
+        <v>276</v>
       </c>
     </row>
     <row r="326" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A326" s="1" t="s">
-        <v>365</v>
+        <v>262</v>
       </c>
       <c r="B326" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="327" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A327" s="1" t="s">
-        <v>366</v>
+        <v>332</v>
       </c>
       <c r="B327" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="328" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A328" s="1" t="s">
-        <v>367</v>
+        <v>258</v>
       </c>
       <c r="B328" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="329" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A329" s="1" t="s">
-        <v>368</v>
+        <v>305</v>
       </c>
       <c r="B329" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="330" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A330" s="1" t="s">
-        <v>369</v>
+        <v>293</v>
       </c>
       <c r="B330" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="331" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A331" s="1" t="s">
-        <v>370</v>
+        <v>295</v>
       </c>
       <c r="B331" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="332" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A332" s="1" t="s">
-        <v>371</v>
+        <v>306</v>
       </c>
       <c r="B332" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="333" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A333" s="1" t="s">
-        <v>372</v>
+        <v>335</v>
       </c>
       <c r="B333" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="334" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A334" s="1" t="s">
-        <v>373</v>
+        <v>259</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="335" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A335" s="1" t="s">
-        <v>374</v>
+        <v>310</v>
       </c>
       <c r="B335" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="336" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A336" s="1" t="s">
-        <v>375</v>
+        <v>336</v>
       </c>
       <c r="B336" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="337" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A337" s="1" t="s">
-        <v>376</v>
+        <v>263</v>
       </c>
       <c r="B337" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="338" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A338" s="1" t="s">
-        <v>377</v>
+        <v>94</v>
       </c>
       <c r="B338" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="339" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A339" s="1" t="s">
-        <v>378</v>
+        <v>337</v>
       </c>
       <c r="B339" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="340" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A340" s="1" t="s">
-        <v>379</v>
+        <v>312</v>
       </c>
       <c r="B340" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="341" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A341" s="1" t="s">
-        <v>380</v>
+        <v>95</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="342" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A342" s="1" t="s">
-        <v>381</v>
+        <v>96</v>
       </c>
       <c r="B342" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="343" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A343" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B343" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="344" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A344" s="1" t="s">
-        <v>383</v>
+        <v>265</v>
       </c>
       <c r="B344" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="345" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A345" s="1" t="s">
-        <v>384</v>
+        <v>266</v>
       </c>
       <c r="B345" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="346" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A346" s="1" t="s">
-        <v>385</v>
+        <v>296</v>
       </c>
       <c r="B346" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="347" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A347" s="1" t="s">
-        <v>386</v>
+        <v>297</v>
       </c>
       <c r="B347" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="348" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A348" s="1" t="s">
-        <v>387</v>
+        <v>298</v>
       </c>
       <c r="B348" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="349" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A349" s="1" t="s">
-        <v>388</v>
+        <v>299</v>
       </c>
       <c r="B349" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="350" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A350" s="1" t="s">
-        <v>389</v>
+        <v>300</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="351" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A351" s="1" t="s">
-        <v>390</v>
+        <v>301</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="352" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A352" s="1" t="s">
-        <v>391</v>
+        <v>302</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="353" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A353" s="1" t="s">
-        <v>392</v>
+        <v>303</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="354" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A354" s="1" t="s">
-        <v>393</v>
+        <v>374</v>
       </c>
       <c r="B354" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="355" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A355" s="1" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="B355" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="356" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A356" s="1" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
       <c r="B356" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="357" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A357" s="1" t="s">
-        <v>396</v>
+        <v>377</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="358" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A358" s="1" t="s">
-        <v>397</v>
+        <v>304</v>
       </c>
       <c r="B358" s="1" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="359" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A359" s="1" t="s">
-        <v>398</v>
+        <v>97</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>180</v>
+        <v>294</v>
       </c>
     </row>
     <row r="360" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A360" s="1" t="s">
-        <v>399</v>
+        <v>267</v>
       </c>
       <c r="B360" s="1" t="s">
-        <v>64</v>
+        <v>294</v>
       </c>
     </row>
     <row r="361" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A361" s="1" t="s">
-        <v>400</v>
+        <v>58</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>224</v>
+        <v>309</v>
       </c>
     </row>
     <row r="362" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A362" s="1" t="s">
-        <v>401</v>
+        <v>328</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>182</v>
+        <v>309</v>
       </c>
     </row>
     <row r="363" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A363" s="1" t="s">
-        <v>402</v>
+        <v>314</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>10</v>
+        <v>309</v>
       </c>
     </row>
     <row r="364" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A364" s="1" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
       <c r="B364" s="1" t="s">
-        <v>180</v>
+        <v>309</v>
       </c>
     </row>
     <row r="365" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A365" s="1" t="s">
-        <v>404</v>
+        <v>253</v>
       </c>
       <c r="B365" s="1" t="s">
-        <v>101</v>
+        <v>309</v>
       </c>
     </row>
     <row r="366" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A366" s="1" t="s">
-        <v>405</v>
+        <v>386</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>332</v>
+        <v>309</v>
       </c>
     </row>
     <row r="367" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A367" s="1" t="s">
-        <v>406</v>
+        <v>327</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
     <row r="368" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A368" s="1" t="s">
-        <v>409</v>
+        <v>316</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>95</v>
+        <v>309</v>
       </c>
     </row>
     <row r="369" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A369" s="1" t="s">
-        <v>410</v>
+        <v>388</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>10</v>
+        <v>318</v>
       </c>
     </row>
     <row r="370" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A370" s="1" t="s">
-        <v>411</v>
+        <v>11</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>182</v>
+        <v>318</v>
       </c>
     </row>
     <row r="371" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A371" s="1" t="s">
-        <v>412</v>
+        <v>319</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>182</v>
+        <v>318</v>
       </c>
     </row>
     <row r="372" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A372" s="1" t="s">
-        <v>413</v>
+        <v>320</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>10</v>
+        <v>318</v>
       </c>
     </row>
     <row r="373" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A373" s="1" t="s">
-        <v>414</v>
+        <v>321</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>224</v>
+        <v>318</v>
       </c>
     </row>
     <row r="374" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A374" s="1" t="s">
-        <v>415</v>
+        <v>322</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="375" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A375" s="1" t="s">
-        <v>416</v>
+        <v>323</v>
       </c>
       <c r="B375" s="1" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="376" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A376" s="1" t="s">
-        <v>417</v>
+        <v>376</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>332</v>
+        <v>318</v>
       </c>
     </row>
     <row r="377" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A377" s="1" t="s">
-        <v>418</v>
+        <v>324</v>
       </c>
       <c r="B377" s="1" t="s">
-        <v>224</v>
+        <v>318</v>
       </c>
     </row>
     <row r="378" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A378" s="1" t="s">
-        <v>419</v>
+        <v>326</v>
       </c>
       <c r="B378" s="1" t="s">
-        <v>224</v>
+        <v>318</v>
       </c>
     </row>
     <row r="379" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A379" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="B379" s="1" t="s">
-        <v>445</v>
+        <v>325</v>
+      </c>
+      <c r="B379" s="3" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="380" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A380" s="1" t="s">
-        <v>421</v>
+        <v>404</v>
       </c>
       <c r="B380" s="1" t="s">
-        <v>444</v>
+        <v>414</v>
       </c>
     </row>
     <row r="381" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A381" s="1" t="s">
-        <v>422</v>
+        <v>405</v>
       </c>
       <c r="B381" s="1" t="s">
-        <v>443</v>
+        <v>414</v>
       </c>
     </row>
     <row r="382" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A382" s="1" t="s">
-        <v>423</v>
+        <v>196</v>
       </c>
       <c r="B382" s="1" t="s">
-        <v>442</v>
+        <v>148</v>
       </c>
     </row>
     <row r="383" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A383" s="1" t="s">
-        <v>424</v>
+        <v>147</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>443</v>
+        <v>148</v>
       </c>
     </row>
     <row r="384" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A384" s="1" t="s">
-        <v>425</v>
+        <v>148</v>
       </c>
       <c r="B384" s="1" t="s">
-        <v>443</v>
+        <v>148</v>
       </c>
     </row>
     <row r="385" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A385" s="1" t="s">
-        <v>426</v>
+        <v>149</v>
       </c>
       <c r="B385" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="386" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A386" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="B386" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="387" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A387" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="B387" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="388" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A388" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="B388" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="389" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A389" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="B389" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="390" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A390" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="B390" s="1" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="391" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A391" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="B391" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="392" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A392" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="B392" s="1" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="393" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A393" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="B393" s="1" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="394" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A394" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="B394" s="1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="395" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A395" s="1" t="s">
-        <v>436</v>
-      </c>
-      <c r="B395" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="396" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A396" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="B396" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="397" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A397" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="B397" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="398" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A398" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="B398" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="399" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A399" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="B399" s="1" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="400" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A400" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="B400" s="1" t="s">
-        <v>443</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12Seite &amp;P</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>